<commit_message>
chore: capture jingji-new local snapshot
</commit_message>
<xml_diff>
--- a/public/templates/竞迹训练数据导入模板.xlsx
+++ b/public/templates/竞迹训练数据导入模板.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="每日训练数据" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="专项测试成绩" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="专项训练成绩" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="填写说明" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -189,13 +189,13 @@
     <t>教练备注</t>
   </si>
   <si>
-    <t>竞迹｜专项距离测试成绩</t>
+    <t>竞迹｜专项距离训练成绩</t>
   </si>
   <si>
     <t>项目必填。赛艇与皮划艇分别形成独立排名；每个运动员或组合占一行，多人艇姓名用“、”分隔。</t>
   </si>
   <si>
-    <t>测试对象</t>
+    <t>训练对象</t>
   </si>
   <si>
     <t>环境条件</t>
@@ -207,10 +207,10 @@
     <t>补充信息</t>
   </si>
   <si>
-    <t>测试日期</t>
-  </si>
-  <si>
-    <t>测试距离(m)</t>
+    <t>训练日期</t>
+  </si>
+  <si>
+    <t>训练距离(m)</t>
   </si>
   <si>
     <t>艇型</t>
@@ -231,7 +231,7 @@
     <t>风向风速</t>
   </si>
   <si>
-    <t>测试地点</t>
+    <t>训练地点</t>
   </si>
   <si>
     <t>历史最好</t>
@@ -288,22 +288,22 @@
     <t>项目必须填写；赛艇与皮划艇数据分别进入各自空间</t>
   </si>
   <si>
-    <t>专项测试成绩</t>
-  </si>
-  <si>
-    <t>250m等专项距离排名与历史比较</t>
-  </si>
-  <si>
-    <t>一个运动员或一个组合的一次测试</t>
-  </si>
-  <si>
-    <t>日期、项目、距离、艇型、组别、姓名、至少一轮</t>
+    <t>专项训练成绩</t>
+  </si>
+  <si>
+    <t>250m等专项距离训练排名与历史比较</t>
+  </si>
+  <si>
+    <t>一个运动员或一个组合的一次训练</t>
+  </si>
+  <si>
+    <t>训练日期、项目、距离、艇型、组别、姓名、至少一轮</t>
   </si>
   <si>
     <t>轮次平均、本次最好、排名、历史最好差值</t>
   </si>
   <si>
-    <t>项目必须填写；同项目同批次重复导入会覆盖</t>
+    <t>项目必须填写；同项目同训练批次重复导入会覆盖</t>
   </si>
   <si>
     <t>成绩格式示例</t>
@@ -3861,7 +3861,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4883,7 +4883,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4995,6 +4995,6 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>